<commit_message>
Polish stock reconciliation skill submission
</commit_message>
<xml_diff>
--- a/outputs/stock_return_reconciliation_demo.xlsx
+++ b/outputs/stock_return_reconciliation_demo.xlsx
@@ -167,10 +167,34 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Security P&amp;L basis</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Sample security P&amp;L is calculated in each security's source currency, then translated to KRW at sell-date FX for realized P&amp;L and as-of FX for unrealized P&amp;L; it is not a historical-FX cost-basis or tax-lot statement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Annualized XIRR note</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Annualized XIRR is a dated cash-flow diagnostic from mock data, not a forecast.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>Boundary</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Not investment, tax, legal, accounting, or trading advice</t>
         </is>

</xml_diff>